<commit_message>
Agregando costos de mercancia 139.888
</commit_message>
<xml_diff>
--- a/Ventas_CJ.xlsx
+++ b/Ventas_CJ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/463e7e6710c11b9a/Algoritmos/negocio de CJ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="11_6FEF09247D2DE7EAAE0E143F64DE01DD4E1F9209" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44FCB161-1329-4D5D-90EC-1EB1BC36BC62}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="11_6FEF09247D2DE7EAAE0E143F64DE01DD4E1F9209" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D91BFB6E-68C3-4467-A102-6D05BDE94AA0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="100">
   <si>
     <t>Fecha</t>
   </si>
@@ -337,6 +337,12 @@
   <si>
     <t xml:space="preserve"> </t>
   </si>
+  <si>
+    <t>5 pantalones old money blancos</t>
+  </si>
+  <si>
+    <t>Renovar Inventario</t>
+  </si>
 </sst>
 </file>
 
@@ -573,15 +579,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -627,6 +624,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -929,7 +933,7 @@
       <c r="H1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="I1" s="43" t="s">
+      <c r="I1" s="40" t="s">
         <v>68</v>
       </c>
     </row>
@@ -957,10 +961,10 @@
         <f t="shared" ref="G2:G56" si="1">IF(A2&lt;&gt;"",MONTH(A2),"")</f>
         <v>9</v>
       </c>
-      <c r="H2" s="42" t="s">
+      <c r="H2" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="I2" s="42" t="s">
+      <c r="I2" s="39" t="s">
         <v>94</v>
       </c>
     </row>
@@ -988,72 +992,72 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H3" s="42" t="s">
+      <c r="H3" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="I3" s="42" t="s">
+      <c r="I3" s="39" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="45">
+      <c r="A4" s="42">
         <v>46281</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="43" t="s">
         <v>89</v>
       </c>
-      <c r="C4" s="47">
+      <c r="C4" s="44">
         <v>34</v>
       </c>
-      <c r="D4" s="47">
+      <c r="D4" s="44">
         <v>2</v>
       </c>
-      <c r="E4" s="48">
+      <c r="E4" s="45">
         <v>95000</v>
       </c>
-      <c r="F4" s="48">
+      <c r="F4" s="45">
         <f t="shared" si="0"/>
         <v>190000</v>
       </c>
-      <c r="G4" s="49">
+      <c r="G4" s="46">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H4" s="50" t="s">
+      <c r="H4" s="47" t="s">
         <v>93</v>
       </c>
-      <c r="I4" s="50" t="s">
+      <c r="I4" s="47" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="45">
+      <c r="A5" s="42">
         <v>46281</v>
       </c>
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="43" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="47" t="s">
+      <c r="C5" s="44" t="s">
         <v>88</v>
       </c>
-      <c r="D5" s="47">
+      <c r="D5" s="44">
         <v>1</v>
       </c>
-      <c r="E5" s="48">
+      <c r="E5" s="45">
         <v>60000</v>
       </c>
-      <c r="F5" s="48">
+      <c r="F5" s="45">
         <f t="shared" si="0"/>
         <v>60000</v>
       </c>
-      <c r="G5" s="49">
+      <c r="G5" s="46">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H5" s="50" t="s">
+      <c r="H5" s="47" t="s">
         <v>93</v>
       </c>
-      <c r="I5" s="50" t="s">
+      <c r="I5" s="47" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1064,7 +1068,7 @@
       <c r="B6" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="C6" s="41" t="s">
         <v>88</v>
       </c>
       <c r="D6" s="7">
@@ -1081,10 +1085,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H6" s="42" t="s">
+      <c r="H6" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="I6" s="42" t="s">
+      <c r="I6" s="39" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1112,10 +1116,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H7" s="42" t="s">
+      <c r="H7" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="I7" s="42" t="s">
+      <c r="I7" s="39" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1126,7 +1130,7 @@
       <c r="B8" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="41" t="s">
         <v>88</v>
       </c>
       <c r="D8" s="7">
@@ -1143,46 +1147,46 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H8" s="42" t="s">
+      <c r="H8" s="39" t="s">
         <v>92</v>
       </c>
-      <c r="I8" s="42" t="s">
+      <c r="I8" s="39" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="45">
+      <c r="A9" s="42">
         <v>46282</v>
       </c>
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="47" t="s">
+      <c r="C9" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="47">
+      <c r="D9" s="44">
         <v>1</v>
       </c>
-      <c r="E9" s="48">
+      <c r="E9" s="45">
         <v>85000</v>
       </c>
-      <c r="F9" s="48">
+      <c r="F9" s="45">
         <f t="shared" si="0"/>
         <v>85000</v>
       </c>
-      <c r="G9" s="49">
+      <c r="G9" s="46">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H9" s="50" t="s">
+      <c r="H9" s="47" t="s">
         <v>92</v>
       </c>
-      <c r="I9" s="50" t="s">
+      <c r="I9" s="47" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="53">
+      <c r="A10" s="50">
         <v>46283</v>
       </c>
       <c r="B10" s="31" t="s">
@@ -1205,15 +1209,15 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H10" s="52" t="s">
+      <c r="H10" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="I10" s="52" t="s">
+      <c r="I10" s="49" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="53">
+      <c r="A11" s="50">
         <v>46283</v>
       </c>
       <c r="B11" s="13" t="s">
@@ -1236,15 +1240,15 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H11" s="52" t="s">
+      <c r="H11" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="I11" s="52" t="s">
+      <c r="I11" s="49" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="53">
+      <c r="A12" s="50">
         <v>46283</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -1267,15 +1271,15 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H12" s="52" t="s">
+      <c r="H12" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="I12" s="52" t="s">
+      <c r="I12" s="49" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="53">
+      <c r="A13" s="50">
         <v>46284</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -1298,15 +1302,15 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H13" s="52" t="s">
+      <c r="H13" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="I13" s="52" t="s">
+      <c r="I13" s="49" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="53">
+      <c r="A14" s="50">
         <v>46284</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -1329,15 +1333,15 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H14" s="52" t="s">
+      <c r="H14" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="I14" s="52" t="s">
+      <c r="I14" s="49" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="53">
+      <c r="A15" s="50">
         <v>46284</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -1360,15 +1364,15 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H15" s="52" t="s">
+      <c r="H15" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="I15" s="52" t="s">
+      <c r="I15" s="49" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="53">
+      <c r="A16" s="50">
         <v>46284</v>
       </c>
       <c r="B16" s="6" t="s">
@@ -1391,10 +1395,10 @@
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="H16" s="52" t="s">
+      <c r="H16" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="I16" s="52" t="s">
+      <c r="I16" s="49" t="s">
         <v>94</v>
       </c>
     </row>
@@ -5556,11 +5560,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="51" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
     </row>
     <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
@@ -6902,7 +6906,7 @@
       </c>
       <c r="B114" s="22">
         <f>SUM(Gastos!D2:D299)</f>
-        <v>27400</v>
+        <v>167288</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.3">
@@ -6911,7 +6915,7 @@
       </c>
       <c r="B115" s="22">
         <f>B113-B114</f>
-        <v>1227600</v>
+        <v>1087712</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -6928,12 +6932,12 @@
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A120" s="24" t="s">
+      <c r="A120" s="54" t="s">
         <v>60</v>
       </c>
       <c r="B120" s="25">
         <f>SUMIFS(Gastos!$D$2:$D$299,Gastos!$B$2:$B$299,A120)</f>
-        <v>0</v>
+        <v>139888</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.3">
@@ -7005,7 +7009,7 @@
       </c>
       <c r="B128" s="27">
         <f>SUM(B120:B127)</f>
-        <v>27400</v>
+        <v>167288</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
@@ -7099,7 +7103,7 @@
       </c>
       <c r="B141" s="25">
         <f>SUMIFS(Gastos!$D$2:$D$299,Gastos!$F$2:$F$299,9)</f>
-        <v>27400</v>
+        <v>167288</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.3">
@@ -7170,23 +7174,23 @@
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="36" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" s="33" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="35" t="s">
+      <c r="C2" s="32" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="33">
+      <c r="D2" s="52">
         <v>46279</v>
       </c>
-      <c r="E2" s="34">
+      <c r="E2" s="53">
         <v>395519</v>
       </c>
-      <c r="F2" s="35" t="s">
+      <c r="F2" s="32" t="s">
         <v>84</v>
       </c>
     </row>
@@ -7194,29 +7198,41 @@
       <c r="A3" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="32" t="s">
         <v>85</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="32" t="s">
         <v>83</v>
       </c>
-      <c r="D3" s="33">
+      <c r="D3" s="52">
         <v>46280</v>
       </c>
-      <c r="E3" s="34">
+      <c r="E3" s="53">
         <v>275904</v>
       </c>
-      <c r="F3" s="35" t="s">
+      <c r="F3" s="32" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="28"/>
+    <row r="4" spans="1:6" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="52">
+        <v>46285</v>
+      </c>
+      <c r="E4" s="53">
+        <v>139888</v>
+      </c>
+      <c r="F4" s="32" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7"/>
@@ -8793,7 +8809,7 @@
       </c>
       <c r="E202" s="10">
         <f>SUMIFS(E2:E199,A2:A199,"Comprado")</f>
-        <v>671423</v>
+        <v>811311</v>
       </c>
     </row>
     <row r="204" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -8848,32 +8864,40 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="40" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38">
+    <row r="2" spans="1:6" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="35">
         <v>46279</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="38" t="s">
         <v>87</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="D2" s="37">
+      <c r="D2" s="34">
         <v>27400</v>
       </c>
-      <c r="F2" s="40">
+      <c r="F2" s="37">
         <f t="shared" ref="F2:F64" si="0">IF(A2&lt;&gt;"",MONTH(A2),"")</f>
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="25"/>
-      <c r="F3" t="str">
+      <c r="A3" s="35">
+        <v>46285</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="36" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="34">
+        <v>139888</v>
+      </c>
+      <c r="F3">
         <f t="shared" si="0"/>
-        <v/>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -11842,7 +11866,7 @@
       </c>
       <c r="D301" s="22">
         <f>SUM(D2:D299)</f>
-        <v>27400</v>
+        <v>167288</v>
       </c>
     </row>
     <row r="303" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>